<commit_message>
added part to bom
</commit_message>
<xml_diff>
--- a/SLSSV3 BoM.xlsx
+++ b/SLSSV3 BoM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://npluk-my.sharepoint.com/personal/james_edwards_npl_co_uk/Documents/Documents/SLSS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edwar\Documents\SLSS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="8_{93ED6D48-6C45-4EA7-9344-3347BCEAFEC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B5F5F2B-6126-4BF8-BA42-A9B8271614E9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{417155C7-FF31-4824-81CF-6BE96CF2BA7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14955" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{0175BE9B-09DB-4935-9617-04C8C213D07E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{0175BE9B-09DB-4935-9617-04C8C213D07E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>No</t>
   </si>
@@ -54,6 +54,18 @@
   </si>
   <si>
     <t>Part number</t>
+  </si>
+  <si>
+    <t>PSU</t>
+  </si>
+  <si>
+    <t>24V 5A PSU brick</t>
+  </si>
+  <si>
+    <t>https://uk.rs-online.com/web/p/ac-dc-adapters/2837427?gb=a</t>
+  </si>
+  <si>
+    <t>283-7427</t>
   </si>
 </sst>
 </file>
@@ -468,6 +480,26 @@
         <v>5</v>
       </c>
     </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" t="s">
+        <v>9</v>
+      </c>
+    </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.35">
       <c r="H7" s="1"/>
     </row>

</xml_diff>